<commit_message>
Feat: Add color in batch content
</commit_message>
<xml_diff>
--- a/test/if-batch-message-flow/output_latest.xlsx
+++ b/test/if-batch-message-flow/output_latest.xlsx
@@ -26,15 +26,21 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFDE9D9"/>
+        <bgColor rgb="FFFDE9D9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,13 +48,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -613,47 +636,47 @@
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>BATCH_START(AccountAudit)</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr"/>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>{"target_user":"admin","from_status":${CONTEXT.last_status}}</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr"/>
-      <c r="E6" s="1" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>START</t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="315" customHeight="1">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>/redfish/v1/AccountService/Accounts/admin</t>
         </is>
       </c>
-      <c r="C7" s="1" t="n"/>
-      <c r="D7" s="1" t="inlineStr">
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>${BATCH.CONTEXT.http_code} = ${STATUSCODE}
 ${BATCH.CONTEXT.user_enabled} = ${RESPONSE.Enabled}</t>
         </is>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="F7" s="1" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>{
     "@odata.id": "/redfish/v1/AccountService/Accounts/admin",
@@ -680,26 +703,26 @@
       </c>
     </row>
     <row r="8" ht="375" customHeight="1">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>/redfish/v1/AccountService</t>
         </is>
       </c>
-      <c r="C8" s="1" t="n"/>
-      <c r="D8" s="1" t="inlineStr">
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>${BATCH.CONTEXT.service_enabled} = ${RESPONSE.ServiceEnabled}</t>
         </is>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="E8" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>{
     "@odata.type": "#AccountService.v1_15_1.AccountService",
@@ -730,24 +753,24 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>BATCH_END(AccountAudit)</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr"/>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>{"target_user":"admin","from_status":${CONTEXT.last_status}}</t>
         </is>
       </c>
-      <c r="D9" s="1" t="inlineStr"/>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
     </row>
     <row r="10" ht="375" customHeight="1">
       <c r="A10" s="1" t="inlineStr">

</xml_diff>